<commit_message>
Correct cheat-sheet Big-O to match implemented solutions
6 levels used textbook-optimal complexity that the in-game code doesn't match:
- bubble-sort: O(n^2) best (no swapped-flag early exit)
- lis: O(n^2) (DP impl, not patience+binary search)
- suffix-array / suffix-array-ds: O(n^2 log n) (naive sorted() of suffix slices)
- lsm-tree: O(n) read (get linearly scans SSTables)
- a-star: O(E log V) worst (explicit graph + heap, degrades to Dijkstra)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/CodeCloze_Cheatsheet.xlsx
+++ b/reference/CodeCloze_Cheatsheet.xlsx
@@ -756,7 +756,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>O(n)</t>
+          <t>O(n^2)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
@@ -3992,7 +3992,7 @@
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>O(n log n)</t>
+          <t>O(n^2)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>O(b^d)</t>
+          <t>O(E log V)</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -6599,17 +6599,17 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>O(n log n)</t>
+          <t>O(n^2 log n)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>O(n log n)</t>
+          <t>O(n^2 log n)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>O(n)</t>
+          <t>O(n^2)</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -10425,7 +10425,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>O(log n) read</t>
+          <t>O(n) read (linear SSTable scan)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -10904,17 +10904,17 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>O(m log n) search</t>
+          <t>O(n^2 log n)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>O(n log n) build</t>
+          <t>O(n^2 log n)</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>O(n)</t>
+          <t>O(n^2)</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">

</xml_diff>